<commit_message>
everything green has been paid for
</commit_message>
<xml_diff>
--- a/BOMs/master_BOM.xlsx
+++ b/BOMs/master_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcoyaipen/Documents/GitHub/RGA_Boards/BOMs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E760B98-A8F6-424A-8382-65E98F857651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E229C4-9E1F-D146-A12C-CF3207BE8005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="235">
   <si>
     <t>Ref</t>
   </si>
@@ -149,9 +149,6 @@
     <t>https://www.google.com/aclk?sa=L&amp;ai=DChsSEwiWusHF-aqTAxVDMggFHTBmMbMYACICCAEQCxoCbWQ&amp;ae=2&amp;co=1&amp;ase=2&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpkjIy16ySTUUYgYVDO6fmXIY_THXMJYLLgxbnnA8Mx3mVvjMK4-nqcaAt3zEALw_wcB&amp;cid=CAAS0gHkaEgvstGWlVoXALWSnP3zED-X5Mk0jxq9rw6e4f0Q7bVVu7A79fwvJzRC74zlt_K3ygvNXyH-UwRAzABR9PJKdFAnolNF-tGndwxSdfJJMSMbwIUky49wRrTY8H_k1gyyDoiDFt83PmA7YO7PrwWAuecgpR2G59eyrvcTZIjH1pE4qUIi2bP0fWRbSczrO6lzYzKkohnyfou_DcmQiB8ighpUGMlaVCpcC7GL56QHb9A2NaWGDbdbLQ4DOc4uFS_iFXJCdFOIJXmrruZU-Rlxkck&amp;cce=2&amp;category=acrcp_v1_71&amp;sig=AOD64_3emY5A5fDU1ffsKevGOIfQUvLVCA&amp;ctype=5&amp;q=&amp;nis=4&amp;ved=2ahUKEwio5LvF-aqTAxV0hIkEHVIsM8oQ5bgDKAB6BAgpEAs&amp;adurl=</t>
   </si>
   <si>
-    <t>https://www.google.com/aclk?sa=L&amp;ai=DChsSEwituPLd-aqTAxUZNwgFHa-GD4gYACICCAEQBxoCbWQ&amp;ae=2&amp;co=1&amp;ase=2&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpmBvJfirg1p6DDHeznVZ9YtKp7ZVF6WzO8CLhBwFgSoU5ys0ucyYp4aAu2DEALw_wcB&amp;cid=CAAS0gHkaAtW7NPcdGhwjEapSxAPVzRINDK53XzUxak0Hw05rAXIlDiIMV1p7QOjULVKKhZa-Qs-d-j_qC5F1YY7hFcj-rkTFjHLymwxjxXPyhUsz1ZxT-rz1DQ5p2eTH9PL6SFQ9OhfwhMy79GcGz8jqLEwgw0TQBZ7B4MBiDhF8R1v_G5nEtIgxcSZ9aGYPqe6Adzn3LQkIxWiiHJeBYaXs-guxAhqOl2rj0SFcMJ4BdKnF0uazOPwtnZczWXMQe7J8VJx6OY9pet2wTPEsQe0OrKBwzs&amp;cce=2&amp;category=acrcp_v1_71&amp;sig=AOD64_2QIyt6r6sLB1GgvNnTusKDQ2WBvw&amp;ctype=5&amp;q=&amp;nis=4&amp;ved=2ahUKEwjFnezd-aqTAxULmYkEHbfwGqAQ5bgDKAB6BAgjEAs&amp;adurl=</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/omron-electronics-inc-emc-div/B3U-1000P/1534338</t>
   </si>
   <si>
@@ -425,9 +422,6 @@
     <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-13100RL/12756438?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpn6BH00nvTHufUr9H_-Hg3WEKvE2bn5P98fg2GflffjclQ8k9-V7k4aAmM_EALw_wcB</t>
   </si>
   <si>
-    <t>https://www.digikey.com/en/products/detail/vishay-dale-thin-film/PNM0603E5002BST5/2120326</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMEF0603FT7K50/16840016?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpnOo1KF7lNez0MbSDEXe3voSS7k8C5CzSx3uagLZW_0-A6xuaswliUaAqm3EALw_wcB</t>
   </si>
   <si>
@@ -446,9 +440,6 @@
     <t>https://www.digikey.com/en/products/detail/molex/0039012020/61315?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20234014242&amp;gbraid=0AAAAADrbLlgAu2bzHcOYngWuQW7ztkGxJ&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpl856nujVS8Geug3cuhZcB4DoCpr9xpRmmPa6mjs7ZFHlpXedxvij0aAkumEALw_wcB</t>
   </si>
   <si>
-    <t>https://www.google.com/aclk?sa=L&amp;ai=DChsSEwji4_jSqKuTAxXbOAgFHeK8OeYYACICCAEQCBoCbWQ&amp;ae=2&amp;co=1&amp;ase=2&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpl-k6ctg8WXehD5UUFDkewhPiu-oilZ4mS4mmlSLGKQBUFXJMNnSXoaAs8aEALw_wcB&amp;cid=CAASugHkaDfxLfEHb4HBnYsrG36tu5hK68e1hCAg8tFT2ZJu8XvUGe6f4Ha3iumyRGIhhF3lDaVUPmVBubz5vAhJWb4-QIbSpAqj8h0OIMstipnlRmWKwB4SArJCSaxMqOv-rfYacAZrKzcLayfiQ6Y47YWtYUId_RlrQRR2AIfCChtU0PP4EKOP0lZXPwO8WaK0YySpKwe-1rizCk75GJssFAvdjc58PLhdBRijeMq4n8exsbeKrLC3Lls9coY&amp;cce=2&amp;category=acrcp_v1_71&amp;sig=AOD64_3Ybiw-eUxoczb4SvanAiK6QXWjwg&amp;ctype=5&amp;q=&amp;nis=4&amp;ved=2ahUKEwi-qvPSqKuTAxU3l4kEHXGaDhsQ5bgDKAB6BAguEBU&amp;adurl=</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
@@ -539,20 +530,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">0.3u </t>
   </si>
   <si>
@@ -650,13 +627,127 @@
   </si>
   <si>
     <t>we will steal from robinson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERA-3AEB333V/1465890</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-07470KL/727257</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERJ-3EKF8201V/1746448</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERA-3AEB123V/1465880</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-07560RL/727304</t>
+  </si>
+  <si>
+    <t>None avaiable on digikey</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603JR-070RL/726675</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMCF0603FT130K/1761272</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603JR-0718KL/726725</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RT0603BRD0740KL/7708329</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMCF0603FT36K0/1713967</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RT0603FRE078K98L/17020100</t>
+  </si>
+  <si>
+    <t>I got 1% 8.98kOhms</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-071ML/726844</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-072KL/727009</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERA-3AEB302V/1465865</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERA-3AEB154V/1465906</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERA-3AEB153V/1465882</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMCF0603FT1K00/1761077</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/vishay-dale/CRCW06032K40FKEA/1174709</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-076K2L/727319</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-07510RL/727285</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/panasonic-electronic-components/ERA-3AEB203V/1465885</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/yageo/RT0603BRD0750KL/7708337</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Is this still 0603?? https://www.digikey.com/en/products/detail/vishay-dale/RCP0603W100RGEB/5481867</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/omron-electronics-inc-emc-div/B3FS-1000/3487234?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20243136172&amp;gbraid=0AAAAADrbLlh8rWNrACXpz8wMlmDvYDuBo&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpmBvJfirg1p6DDHeznVZ9YtKp7ZVF6WzO8CLhBwFgSoU5ys0ucyYp4aAu2DEALw_wcB</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/TS12A12511DCNR/2328661?s=N4IgTCBcDaICoGUCMYCCKCsSkBEDCAcgEogC6AvkA</t>
+  </si>
+  <si>
+    <t>We alreadty have spare from digicorder</t>
+  </si>
+  <si>
+    <t>If we need more we take from shop no?</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/TPL0501-100DCNR/2755770?s=N4IgTCBcDaICoAUAyAGArCgjAWkylAIgMIByASiALoC%2BQA</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/texas-instruments/LM2940IMP-9-0-NOPB/363894?s=N4IgTCBcDaIDIFkwE4AsAGAkggCgWmQDp0B6AOQHkcAhEAXQF8g</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/ADP7118AUJZ-4-5-R7/6599734?s=N4IgTCBcDaIIIBEAKB2AjGgHHAqgKQC0BaAFgDoBWIgJRRAF0BfIA</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/AD8400ARZ1/751162</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/ADA4522-2ARMZ-R7/5268023?s=N4IgTCBcDaIIIBE4BYCsYwFoxwEoFkAtTXAdhAF0BfIA</t>
+  </si>
+  <si>
+    <t>gulp</t>
+  </si>
+  <si>
+    <t>https://www.google.com/aclk?sa=L&amp;ai=DChsSEwji4_jSqKuTAxXbOAgFHeK8OeYYACICCAEQCBoCbWQ&amp;ae=2&amp;co=1&amp;ase=2&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpl-k6ctg8WXehD5UUFDkewhPiu-oilZ4mS4mmlSLGKQBUFXJMNnSXoaAs8aEALw_wcB&amp;cid=CAASugHkaDfxLfEHb4HBnYsrG36tu5hK68e1hCAg8tFT2ZJu8XvUGe6f4Ha3iumyRGIhhF3lDaVUPmVBubz5vAhJWb4-QIbSpAqj8h0OIMstipnlRmWKwB4SArJCSaxMqOv-atype=5&amp;q=&amp;nis=4&amp;ved=2ahUKEwi-qvPSqKuTAxU3l4kEHXGaDhsQ5bgDKAB6BAguEBU&amp;adurl=</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/molex/0436450310/7062847?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20234014242&amp;gbraid=0AAAAADrbLlgAu2bzHcOYngWuQW7ztkGxJ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -706,12 +797,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri (Body)"/>
     </font>
   </fonts>
   <fills count="6">
@@ -810,10 +895,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D394BD76-92DA-4E8D-B179-449D1F8765B5}" name="Table1" displayName="Table1" ref="A15:F140" totalsRowShown="0" headerRowBorderDxfId="0">
-  <autoFilter ref="A15:F140" xr:uid="{D394BD76-92DA-4E8D-B179-449D1F8765B5}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A16:E136">
-    <sortCondition ref="A15:A136"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D394BD76-92DA-4E8D-B179-449D1F8765B5}" name="Table1" displayName="Table1" ref="A15:F141" totalsRowShown="0" headerRowBorderDxfId="0">
+  <autoFilter ref="A15:F141" xr:uid="{D394BD76-92DA-4E8D-B179-449D1F8765B5}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A16:E137">
+    <sortCondition ref="A15:A137"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8644B3C5-A7EF-4556-8A18-B599100B2DB0}" name="Ref"/>
@@ -1090,7 +1175,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A9:F140"/>
+  <dimension ref="A9:F141"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="30.5" customWidth="1"/>
@@ -1102,7 +1187,7 @@
   <sheetData>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B9" s="4"/>
     </row>
@@ -1111,7 +1196,7 @@
         <v>0</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>1</v>
@@ -1123,12 +1208,12 @@
         <v>3</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B16" s="6">
         <v>100</v>
@@ -1140,15 +1225,15 @@
         <v>6</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B17" s="6">
         <v>10</v>
@@ -1160,15 +1245,15 @@
         <v>8</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B18" s="6">
         <v>10</v>
@@ -1177,52 +1262,52 @@
         <v>3</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C19" s="7">
         <v>1</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C20" s="6">
         <v>1</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B21" s="6">
         <v>3</v>
@@ -1231,18 +1316,18 @@
         <v>1</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B22" s="6">
         <v>10</v>
@@ -1251,18 +1336,18 @@
         <v>2</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B23" s="9">
         <v>3</v>
@@ -1271,18 +1356,18 @@
         <v>1</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B24" s="9">
         <v>3</v>
@@ -1291,18 +1376,18 @@
         <v>1</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B25" s="9">
         <v>10</v>
@@ -1311,18 +1396,18 @@
         <v>2</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B26" s="9">
         <v>10</v>
@@ -1331,18 +1416,18 @@
         <v>1</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="27" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B27" s="6">
         <v>10</v>
@@ -1351,18 +1436,18 @@
         <v>1</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="28" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B28" s="9">
         <v>10</v>
@@ -1371,18 +1456,18 @@
         <v>1</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="29" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B29" s="6">
         <v>10</v>
@@ -1391,18 +1476,18 @@
         <v>1</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B30" s="6">
         <v>10</v>
@@ -1411,18 +1496,18 @@
         <v>1</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B31" s="6">
         <v>10</v>
@@ -1431,21 +1516,21 @@
         <v>1</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="32" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C32" s="6">
         <v>37</v>
@@ -1457,12 +1542,12 @@
         <v>26</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="33" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B33" s="7">
         <v>2</v>
@@ -1471,18 +1556,18 @@
         <v>5</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="34" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B34" s="6">
         <v>12</v>
@@ -1497,12 +1582,12 @@
         <v>27</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="35" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B35" s="6">
         <v>50</v>
@@ -1514,15 +1599,15 @@
         <v>5</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B36" s="6">
         <v>10</v>
@@ -1531,18 +1616,18 @@
         <v>4</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="37" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B37" s="6">
         <v>12</v>
@@ -1551,18 +1636,18 @@
         <v>6</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="38" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B38" s="6">
         <v>5</v>
@@ -1571,32 +1656,32 @@
         <v>2</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>28</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="39" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C39" s="6">
         <v>3</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="40" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B40" s="6">
         <v>14</v>
@@ -1605,18 +1690,18 @@
         <v>7</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="41" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B41" s="6">
         <v>10</v>
@@ -1625,18 +1710,18 @@
         <v>2</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="42" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B42" s="6">
         <v>2</v>
@@ -1645,13 +1730,13 @@
         <v>1</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -1662,18 +1747,18 @@
         <v>11</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="44" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B44" s="6">
         <v>24</v>
@@ -1682,18 +1767,18 @@
         <v>11</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>29</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="45" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B45" s="6">
         <v>6</v>
@@ -1705,15 +1790,15 @@
         <v>9</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B46" s="6">
         <v>8</v>
@@ -1722,13 +1807,13 @@
         <v>4</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="47" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -1739,18 +1824,18 @@
         <v>4</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B48" s="6">
         <v>2</v>
@@ -1762,15 +1847,15 @@
         <v>10</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C49" s="7">
         <v>1</v>
@@ -1779,26 +1864,26 @@
         <v>11</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C50">
         <v>3</v>
       </c>
       <c r="D50" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F50" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B51" s="9">
         <v>2</v>
@@ -1810,15 +1895,15 @@
         <v>39281023</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="F51" s="9" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="52" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B52" s="6">
         <v>4</v>
@@ -1830,10 +1915,10 @@
         <v>2068320801</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="53" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -1847,1275 +1932,1532 @@
         <v>2064610800</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B54" s="3"/>
       <c r="C54" s="3">
         <v>1</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="55" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C55" s="7">
         <v>1</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="56" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C56" s="7">
         <v>2</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F56" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="57" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C57" s="7">
         <v>1</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="58" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C58" s="7">
         <v>1</v>
       </c>
       <c r="D58" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A59" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B59" s="6">
+        <v>3</v>
+      </c>
+      <c r="C59" s="6">
+        <v>1</v>
+      </c>
+      <c r="D59" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E58" s="7" t="s">
+      <c r="E59" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F58" s="7" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C59" s="7">
-        <v>1</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="F59" s="7" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A60" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C60" s="7">
-        <v>1</v>
-      </c>
-      <c r="D60" s="7" t="s">
+      <c r="F59" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B60" s="6">
+        <v>2</v>
+      </c>
+      <c r="C60" s="6">
+        <v>1</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="B61" s="6">
+        <v>10</v>
+      </c>
+      <c r="C61" s="6">
+        <v>5</v>
+      </c>
+      <c r="D61" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="E60" s="7" t="s">
+      <c r="E61" s="6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B62" s="6">
+        <v>10</v>
+      </c>
+      <c r="C62" s="6">
+        <v>5</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E62" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="F60" s="7" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A61" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C61" s="7">
-        <v>5</v>
-      </c>
-      <c r="D61" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="E61" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="F61" s="7" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A62" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="C62" s="9">
+      <c r="F62" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A63" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C63" s="9">
         <v>3</v>
       </c>
-      <c r="D62" s="9" t="s">
+      <c r="D63" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F62" s="9" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A63" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="B63" s="6">
-        <v>1</v>
-      </c>
-      <c r="C63" s="6">
-        <v>1</v>
-      </c>
-      <c r="D63" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="F63" s="6" t="s">
-        <v>166</v>
+      <c r="F63" s="9" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="64" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="6" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B64" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C64" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="65" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B65" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>105</v>
+        <v>191</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="66" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B66" s="6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C66" s="6">
+        <v>1</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A67" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B67" s="6">
+        <v>10</v>
+      </c>
+      <c r="C67" s="6">
         <v>5</v>
       </c>
-      <c r="D66" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A67" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="C67" s="9">
+      <c r="D67" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A68" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C68" s="9">
         <v>2</v>
       </c>
-      <c r="D67" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="F67" s="9" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3">
+      <c r="D68" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="F68" s="9" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B69" s="3"/>
+      <c r="C69" s="3">
         <v>4</v>
       </c>
-      <c r="D68" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E68" s="3"/>
-      <c r="F68" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A69" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="B69" s="6">
+      <c r="D69" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="B70" s="6">
         <v>2</v>
       </c>
-      <c r="C69" s="6">
-        <v>1</v>
-      </c>
-      <c r="D69" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E69" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="F69" s="6" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A70" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="C70" s="9">
-        <v>2</v>
-      </c>
-      <c r="D70" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="F70" s="9" t="s">
-        <v>200</v>
+      <c r="C70" s="6">
+        <v>1</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="71" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="9" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C71" s="9">
         <v>2</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F71" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A72" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="C72" s="9">
+        <v>2</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="F72" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A73" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C73" s="7">
+        <v>1</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F73" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B74" s="6">
+        <v>10</v>
+      </c>
+      <c r="C74" s="6">
+        <v>3</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A75" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B75" s="6">
+        <v>10</v>
+      </c>
+      <c r="C75" s="6">
+        <v>4</v>
+      </c>
+      <c r="D75" s="6">
+        <v>440</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A76" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B76" s="6">
+        <v>10</v>
+      </c>
+      <c r="C76" s="6">
+        <v>1</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A77" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B77" s="6">
+        <v>10</v>
+      </c>
+      <c r="C77" s="6">
+        <v>3</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A78" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B78" s="6">
+        <v>10</v>
+      </c>
+      <c r="C78" s="6">
+        <v>2</v>
+      </c>
+      <c r="D78" s="6">
+        <v>240</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A79" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B79" s="6">
+        <v>25</v>
+      </c>
+      <c r="C79" s="6">
+        <v>9</v>
+      </c>
+      <c r="D79" s="6">
+        <v>150</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A80" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B80" s="6">
+        <v>50</v>
+      </c>
+      <c r="C80" s="6">
+        <v>17</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A81" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B81" s="6">
+        <v>10</v>
+      </c>
+      <c r="C81" s="6">
+        <v>3</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A82" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B82" s="6">
+        <v>10</v>
+      </c>
+      <c r="C82" s="6">
+        <v>4</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A83" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B83" s="6">
+        <v>10</v>
+      </c>
+      <c r="C83" s="6">
+        <v>2</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E83" s="6" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A72" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="C72" s="7">
-        <v>1</v>
-      </c>
-      <c r="D72" s="7" t="s">
+      <c r="F83" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A84" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B84" s="6">
+        <v>10</v>
+      </c>
+      <c r="C84" s="6">
+        <v>4</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A85" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B85" s="6">
+        <v>10</v>
+      </c>
+      <c r="C85" s="6">
+        <v>1</v>
+      </c>
+      <c r="D85" s="6">
+        <v>560</v>
+      </c>
+      <c r="E85" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="F85" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A86" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C86" s="7">
+        <v>4</v>
+      </c>
+      <c r="D86" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F86" s="7" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A87" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="C87" s="9">
+        <v>2</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F87" s="9" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A88" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B88" s="6">
+        <v>10</v>
+      </c>
+      <c r="C88" s="6">
+        <v>4</v>
+      </c>
+      <c r="D88" s="6">
+        <v>0</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="F88" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A89" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B89" s="6">
+        <v>10</v>
+      </c>
+      <c r="C89" s="6">
+        <v>1</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F89" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A90" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B90" s="6">
+        <v>10</v>
+      </c>
+      <c r="C90" s="6">
+        <v>1</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="F90" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A91" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B91" s="6">
+        <v>10</v>
+      </c>
+      <c r="C91" s="6">
+        <v>1</v>
+      </c>
+      <c r="D91" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E91" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="F91" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A92" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B92" s="6">
+        <v>10</v>
+      </c>
+      <c r="C92" s="6">
+        <v>1</v>
+      </c>
+      <c r="D92" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A93" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B93" s="6">
+        <v>10</v>
+      </c>
+      <c r="C93" s="6">
+        <v>2</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E93" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="F93" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A94" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B94" s="6">
+        <v>10</v>
+      </c>
+      <c r="C94" s="6">
+        <v>4</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="F94" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A95" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B95" s="6">
+        <v>10</v>
+      </c>
+      <c r="C95" s="6">
+        <v>2</v>
+      </c>
+      <c r="D95" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="F72" s="7" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>68</v>
-      </c>
-      <c r="C73">
+      <c r="E95" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="F95" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A96" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B96" s="6">
+        <v>10</v>
+      </c>
+      <c r="C96" s="6">
+        <v>1</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="F96" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A97" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B97" s="6">
+        <v>10</v>
+      </c>
+      <c r="C97" s="6">
+        <v>1</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="F97" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A98" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B98" s="6">
+        <v>10</v>
+      </c>
+      <c r="C98" s="6">
+        <v>1</v>
+      </c>
+      <c r="D98" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E98" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="F98" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A99" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B99" s="6">
+        <v>25</v>
+      </c>
+      <c r="C99" s="6">
+        <v>12</v>
+      </c>
+      <c r="D99" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="F99" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A100" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B100" s="6">
+        <v>10</v>
+      </c>
+      <c r="C100" s="6">
+        <v>1</v>
+      </c>
+      <c r="D100" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E100" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="F100" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A101" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B101" s="6">
+        <v>10</v>
+      </c>
+      <c r="C101" s="6">
+        <v>5</v>
+      </c>
+      <c r="D101" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="F101" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A102" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B102" s="6">
+        <v>25</v>
+      </c>
+      <c r="C102" s="6">
+        <v>8</v>
+      </c>
+      <c r="D102" s="6">
+        <v>510</v>
+      </c>
+      <c r="E102" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="F102" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A103" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B103" s="6">
+        <v>10</v>
+      </c>
+      <c r="C103" s="6">
         <v>3</v>
       </c>
-      <c r="D73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E73" t="s">
-        <v>30</v>
-      </c>
-      <c r="F73" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>68</v>
-      </c>
-      <c r="C74">
+      <c r="D103" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="F103" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A104" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B104" s="6">
+        <v>8</v>
+      </c>
+      <c r="C104" s="6">
         <v>4</v>
       </c>
-      <c r="D74">
-        <v>440</v>
-      </c>
-      <c r="E74" t="s">
-        <v>31</v>
-      </c>
-      <c r="F74" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>68</v>
-      </c>
-      <c r="C75">
-        <v>1</v>
-      </c>
-      <c r="D75" t="s">
-        <v>13</v>
-      </c>
-      <c r="E75" t="s">
-        <v>32</v>
-      </c>
-      <c r="F75" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>68</v>
-      </c>
-      <c r="C76">
+      <c r="D104" s="6">
+        <v>4.7</v>
+      </c>
+      <c r="E104" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="F104" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A105" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B105" s="6">
+        <v>10</v>
+      </c>
+      <c r="C105" s="6">
+        <v>1</v>
+      </c>
+      <c r="D105" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="E105" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F105" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A106" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B106" s="6">
+        <v>25</v>
+      </c>
+      <c r="C106" s="6">
+        <v>7</v>
+      </c>
+      <c r="D106" s="6">
+        <v>100</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F106" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A107" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B107" s="6">
+        <v>10</v>
+      </c>
+      <c r="C107" s="6">
+        <v>1</v>
+      </c>
+      <c r="D107" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E107" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F107" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A108" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B108" s="6">
+        <v>10</v>
+      </c>
+      <c r="C108" s="6">
+        <v>4</v>
+      </c>
+      <c r="D108" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E108" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="F108" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A109" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B109" s="6">
+        <v>10</v>
+      </c>
+      <c r="C109" s="6">
         <v>3</v>
       </c>
-      <c r="D76" t="s">
-        <v>14</v>
-      </c>
-      <c r="E76" t="s">
-        <v>33</v>
-      </c>
-      <c r="F76" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>68</v>
-      </c>
-      <c r="C77">
+      <c r="D109" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E109" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F109" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A110" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B110" s="6">
+        <v>25</v>
+      </c>
+      <c r="C110" s="6">
+        <v>9</v>
+      </c>
+      <c r="D110" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E110" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="F110" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A111" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="B111" s="9">
+        <v>4</v>
+      </c>
+      <c r="C111" s="9">
         <v>2</v>
       </c>
-      <c r="D77">
-        <v>240</v>
-      </c>
-      <c r="E77" t="s">
-        <v>34</v>
-      </c>
-      <c r="F77" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
-        <v>68</v>
-      </c>
-      <c r="C78">
-        <v>9</v>
-      </c>
-      <c r="D78">
-        <v>150</v>
-      </c>
-      <c r="E78" t="s">
-        <v>35</v>
-      </c>
-      <c r="F78" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>68</v>
-      </c>
-      <c r="C79">
-        <v>17</v>
-      </c>
-      <c r="D79" t="s">
-        <v>15</v>
-      </c>
-      <c r="E79" t="s">
-        <v>36</v>
-      </c>
-      <c r="F79" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>68</v>
-      </c>
-      <c r="C80">
-        <v>3</v>
-      </c>
-      <c r="D80" t="s">
-        <v>52</v>
-      </c>
-      <c r="F80" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>68</v>
-      </c>
-      <c r="C81">
-        <v>4</v>
-      </c>
-      <c r="D81" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>68</v>
-      </c>
-      <c r="C82">
-        <v>2</v>
-      </c>
-      <c r="D82" t="s">
-        <v>55</v>
-      </c>
-      <c r="F82" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
-        <v>68</v>
-      </c>
-      <c r="C83">
-        <v>4</v>
-      </c>
-      <c r="D83" t="s">
-        <v>56</v>
-      </c>
-      <c r="F83" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>68</v>
-      </c>
-      <c r="C84">
-        <v>1</v>
-      </c>
-      <c r="D84">
-        <v>560</v>
-      </c>
-      <c r="F84" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>68</v>
-      </c>
-      <c r="C85">
-        <v>4</v>
-      </c>
-      <c r="D85" t="s">
-        <v>59</v>
-      </c>
-      <c r="F85" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>68</v>
-      </c>
-      <c r="C86">
-        <v>2</v>
-      </c>
-      <c r="D86" t="s">
-        <v>68</v>
-      </c>
-      <c r="F86" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>68</v>
-      </c>
-      <c r="C87">
-        <v>4</v>
-      </c>
-      <c r="D87">
-        <v>0</v>
-      </c>
-      <c r="F87" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>68</v>
-      </c>
-      <c r="C88">
-        <v>1</v>
-      </c>
-      <c r="D88" t="s">
-        <v>75</v>
-      </c>
-      <c r="F88" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
-        <v>68</v>
-      </c>
-      <c r="C89">
-        <v>1</v>
-      </c>
-      <c r="D89" t="s">
-        <v>76</v>
-      </c>
-      <c r="F89" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>68</v>
-      </c>
-      <c r="C90">
-        <v>1</v>
-      </c>
-      <c r="D90" t="s">
-        <v>77</v>
-      </c>
-      <c r="F90" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>68</v>
-      </c>
-      <c r="C91">
-        <v>1</v>
-      </c>
-      <c r="D91" t="s">
-        <v>78</v>
-      </c>
-      <c r="F91" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>68</v>
-      </c>
-      <c r="C92">
-        <v>2</v>
-      </c>
-      <c r="D92" t="s">
-        <v>80</v>
-      </c>
-      <c r="F92" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>68</v>
-      </c>
-      <c r="C93">
-        <v>4</v>
-      </c>
-      <c r="D93" t="s">
-        <v>73</v>
-      </c>
-      <c r="F93" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>68</v>
-      </c>
-      <c r="C94">
-        <v>2</v>
-      </c>
-      <c r="D94" t="s">
-        <v>84</v>
-      </c>
-      <c r="F94" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>68</v>
-      </c>
-      <c r="C95">
-        <v>1</v>
-      </c>
-      <c r="D95" t="s">
-        <v>85</v>
-      </c>
-      <c r="F95" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
-        <v>68</v>
-      </c>
-      <c r="C96">
-        <v>1</v>
-      </c>
-      <c r="D96" t="s">
-        <v>86</v>
-      </c>
-      <c r="F96" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
-        <v>68</v>
-      </c>
-      <c r="C97">
-        <v>1</v>
-      </c>
-      <c r="D97" t="s">
-        <v>87</v>
-      </c>
-      <c r="F97" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>68</v>
-      </c>
-      <c r="C98">
-        <v>12</v>
-      </c>
-      <c r="D98" t="s">
-        <v>74</v>
-      </c>
-      <c r="F98" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
-        <v>68</v>
-      </c>
-      <c r="C99">
-        <v>1</v>
-      </c>
-      <c r="D99" t="s">
-        <v>88</v>
-      </c>
-      <c r="F99" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
-        <v>68</v>
-      </c>
-      <c r="C100">
-        <v>5</v>
-      </c>
-      <c r="D100" t="s">
-        <v>79</v>
-      </c>
-      <c r="F100" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
-        <v>68</v>
-      </c>
-      <c r="C101">
-        <v>8</v>
-      </c>
-      <c r="D101">
-        <v>510</v>
-      </c>
-      <c r="F101" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
-        <v>68</v>
-      </c>
-      <c r="C102">
-        <v>3</v>
-      </c>
-      <c r="D102" t="s">
-        <v>58</v>
-      </c>
-      <c r="F102" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>68</v>
-      </c>
-      <c r="C103">
-        <v>4</v>
-      </c>
-      <c r="D103">
-        <v>4.7</v>
-      </c>
-      <c r="E103" t="s">
-        <v>149</v>
-      </c>
-      <c r="F103" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
-        <v>68</v>
-      </c>
-      <c r="C104">
-        <v>1</v>
-      </c>
-      <c r="D104" t="s">
-        <v>115</v>
-      </c>
-      <c r="E104" t="s">
-        <v>127</v>
-      </c>
-      <c r="F104" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>68</v>
-      </c>
-      <c r="C105">
-        <v>7</v>
-      </c>
-      <c r="D105">
+      <c r="D111" s="9">
         <v>100</v>
       </c>
-      <c r="E105" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="F105" s="2" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
-        <v>68</v>
-      </c>
-      <c r="C106">
-        <v>1</v>
-      </c>
-      <c r="D106" t="s">
-        <v>116</v>
-      </c>
-      <c r="E106" t="s">
-        <v>129</v>
-      </c>
-      <c r="F106" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
-        <v>68</v>
-      </c>
-      <c r="C107">
-        <v>4</v>
-      </c>
-      <c r="D107" t="s">
-        <v>117</v>
-      </c>
-      <c r="E107" t="s">
-        <v>130</v>
-      </c>
-      <c r="F107" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
-        <v>68</v>
-      </c>
-      <c r="C108">
-        <v>3</v>
-      </c>
-      <c r="D108" t="s">
-        <v>57</v>
-      </c>
-      <c r="E108" t="s">
-        <v>131</v>
-      </c>
-      <c r="F108" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
-        <v>68</v>
-      </c>
-      <c r="C109">
-        <v>9</v>
-      </c>
-      <c r="D109" t="s">
-        <v>53</v>
-      </c>
-      <c r="E109" t="s">
-        <v>132</v>
-      </c>
-      <c r="F109" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
-        <v>68</v>
-      </c>
-      <c r="C110">
-        <v>2</v>
-      </c>
-      <c r="D110">
-        <v>100</v>
-      </c>
-      <c r="E110" t="s">
-        <v>150</v>
-      </c>
-      <c r="F110" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
-        <v>140</v>
-      </c>
-      <c r="C111">
-        <v>1</v>
-      </c>
-      <c r="D111" t="s">
-        <v>17</v>
-      </c>
-      <c r="F111" t="s">
-        <v>166</v>
+      <c r="E111" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="F111" s="9" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C112">
         <v>1</v>
       </c>
       <c r="D112" t="s">
+        <v>17</v>
+      </c>
+      <c r="F112" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A113" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B113" s="6">
+        <v>3</v>
+      </c>
+      <c r="C113" s="6">
+        <v>1</v>
+      </c>
+      <c r="D113" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E112" t="s">
-        <v>37</v>
-      </c>
-      <c r="F112" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
-        <v>140</v>
-      </c>
-      <c r="C113">
-        <v>1</v>
-      </c>
-      <c r="D113" t="s">
-        <v>19</v>
-      </c>
-      <c r="F113" t="s">
-        <v>166</v>
+      <c r="E113" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="F113" s="6" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C114">
         <v>1</v>
       </c>
       <c r="D114" t="s">
+        <v>19</v>
+      </c>
+      <c r="F114" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A115" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B115" s="6">
+        <v>3</v>
+      </c>
+      <c r="C115" s="6">
+        <v>1</v>
+      </c>
+      <c r="D115" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E114" t="s">
+      <c r="E115" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F115" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A116" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B116" s="6">
+        <v>10</v>
+      </c>
+      <c r="C116" s="6">
+        <v>9</v>
+      </c>
+      <c r="D116" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E116" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="F116" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A117" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B117" s="6">
+        <v>2</v>
+      </c>
+      <c r="C117" s="6">
+        <v>1</v>
+      </c>
+      <c r="D117" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E117" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F114" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
-        <v>141</v>
-      </c>
-      <c r="C115">
-        <v>9</v>
-      </c>
-      <c r="D115" t="s">
-        <v>21</v>
-      </c>
-      <c r="F115" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
-        <v>141</v>
-      </c>
-      <c r="C116">
-        <v>1</v>
-      </c>
-      <c r="D116" t="s">
-        <v>22</v>
-      </c>
-      <c r="E116" t="s">
+      <c r="F117" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A118" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B118" s="6">
+        <v>1</v>
+      </c>
+      <c r="C118" s="6">
+        <v>1</v>
+      </c>
+      <c r="D118" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E118" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F116" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
-        <v>141</v>
-      </c>
-      <c r="C117">
-        <v>1</v>
-      </c>
-      <c r="D117" t="s">
-        <v>23</v>
-      </c>
-      <c r="E117" t="s">
+      <c r="F118" s="6" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A119" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B119" s="6">
+        <v>10</v>
+      </c>
+      <c r="C119" s="6">
+        <v>3</v>
+      </c>
+      <c r="D119" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E119" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F117" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
-        <v>141</v>
-      </c>
-      <c r="C118">
-        <v>3</v>
-      </c>
-      <c r="D118" t="s">
-        <v>24</v>
-      </c>
-      <c r="E118" t="s">
+      <c r="F119" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A120" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B120" s="6">
+        <v>1</v>
+      </c>
+      <c r="C120" s="6">
+        <v>1</v>
+      </c>
+      <c r="D120" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E120" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F118" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
-        <v>141</v>
-      </c>
-      <c r="C119">
-        <v>1</v>
-      </c>
-      <c r="D119" t="s">
-        <v>25</v>
-      </c>
-      <c r="E119" t="s">
-        <v>42</v>
-      </c>
-      <c r="F119" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
-        <v>141</v>
-      </c>
-      <c r="C120">
+      <c r="F120" s="9" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A121" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B121" s="6">
+        <v>10</v>
+      </c>
+      <c r="C121" s="6">
         <v>4</v>
       </c>
-      <c r="D120" t="s">
-        <v>60</v>
-      </c>
-      <c r="F120" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A121" t="s">
-        <v>141</v>
-      </c>
-      <c r="C121">
+      <c r="D121" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E121" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="F121" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A122" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B122" s="6">
+        <v>4</v>
+      </c>
+      <c r="C122" s="6">
         <v>2</v>
       </c>
-      <c r="D121" t="s">
+      <c r="D122" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E122" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="F122" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A123" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B123" s="6">
+        <v>2</v>
+      </c>
+      <c r="C123" s="6">
+        <v>1</v>
+      </c>
+      <c r="D123" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="F121" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
-        <v>141</v>
-      </c>
-      <c r="C122">
-        <v>1</v>
-      </c>
-      <c r="D122" t="s">
-        <v>63</v>
-      </c>
-      <c r="F122" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A123" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B123" s="5"/>
-      <c r="C123" s="5">
-        <v>1</v>
-      </c>
-      <c r="D123" s="5" t="s">
+      <c r="E123" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="F123" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A124" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="B124" s="5"/>
+      <c r="C124" s="5">
+        <v>1</v>
+      </c>
+      <c r="D124" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E124" s="5"/>
+      <c r="F124" s="5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A125" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B125" s="3"/>
+      <c r="C125" s="3">
+        <v>1</v>
+      </c>
+      <c r="D125" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E123" s="5"/>
-      <c r="F123" s="5" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A124" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B124" s="3"/>
-      <c r="C124" s="3">
-        <v>1</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E124" s="3"/>
-      <c r="F124" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
-        <v>141</v>
-      </c>
-      <c r="C125">
-        <v>1</v>
-      </c>
-      <c r="D125" t="s">
-        <v>81</v>
-      </c>
-      <c r="F125" t="s">
-        <v>166</v>
+      <c r="E125" s="3"/>
+      <c r="F125" s="3" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C126">
         <v>1</v>
       </c>
       <c r="D126" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F126" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
-        <v>141</v>
-      </c>
-      <c r="C127">
-        <v>1</v>
-      </c>
-      <c r="D127" t="s">
-        <v>89</v>
-      </c>
-      <c r="F127" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A127" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B127" s="6">
+        <v>2</v>
+      </c>
+      <c r="C127" s="6">
+        <v>1</v>
+      </c>
+      <c r="D127" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="E127" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="F127" s="6" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C128">
+        <v>1</v>
+      </c>
+      <c r="D128" t="s">
+        <v>88</v>
+      </c>
+      <c r="F128" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A129" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B129" s="6">
+        <v>4</v>
+      </c>
+      <c r="C129" s="6">
         <v>2</v>
       </c>
-      <c r="D128" t="s">
-        <v>96</v>
-      </c>
-      <c r="F128" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
-        <v>141</v>
-      </c>
-      <c r="C129">
-        <v>1</v>
-      </c>
-      <c r="D129" t="s">
-        <v>101</v>
-      </c>
-      <c r="E129" t="s">
-        <v>106</v>
-      </c>
-      <c r="F129" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
-        <v>141</v>
-      </c>
-      <c r="C130">
+      <c r="D129" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E129" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="F129" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A130" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B130" s="6">
+        <v>1</v>
+      </c>
+      <c r="C130" s="6">
+        <v>1</v>
+      </c>
+      <c r="D130" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E130" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F130" s="6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A131" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B131" s="6">
+        <v>41</v>
+      </c>
+      <c r="C131" s="6">
         <v>20</v>
       </c>
-      <c r="D130" t="s">
-        <v>61</v>
-      </c>
-      <c r="E130" t="s">
-        <v>133</v>
-      </c>
-      <c r="F130" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
-        <v>141</v>
-      </c>
-      <c r="C131">
-        <v>1</v>
-      </c>
-      <c r="D131" t="s">
-        <v>118</v>
-      </c>
-      <c r="E131" t="s">
-        <v>134</v>
-      </c>
-      <c r="F131" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="F132" t="s">
-        <v>166</v>
+      <c r="D131" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E131" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F131" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A132" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B132" s="6">
+        <v>2</v>
+      </c>
+      <c r="C132" s="6">
+        <v>1</v>
+      </c>
+      <c r="D132" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="E132" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F132" s="6" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F133" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F134" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E135" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="F135" s="2" t="s">
-        <v>166</v>
+      <c r="F135" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="E136" t="s">
-        <v>136</v>
-      </c>
-      <c r="F136" t="s">
-        <v>166</v>
+      <c r="E136" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E137" s="2" t="s">
+        <v>233</v>
+      </c>
       <c r="F137" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F138" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F139" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F140" t="s">
-        <v>166</v>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F141" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E135" r:id="rId1" display="https://www.digikey.com/en/products/detail/molex/0039012020/61315?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20234014242&amp;gbraid=0AAAAADrbLlgAu2bzHcOYngWuQW7ztkGxJ&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpl856nujVS8Geug3cuhZcB4DoCpr9xpRmmPa6mjs7ZFHlpXedxvij0aAkumEALw_wcB" xr:uid="{7942DB98-5E6F-4A35-88A4-8452DAD088A7}"/>
-    <hyperlink ref="E105" r:id="rId2" display="https://www.digikey.com/en/products/detail/yageo/RC0603FR-13100RL/12756438?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpn6BH00nvTHufUr9H_-Hg3WEKvE2bn5P98fg2GflffjclQ8k9-V7k4aAmM_EALw_wcB" xr:uid="{CA0412C4-4416-4D1B-B39B-A6DED7EA58CF}"/>
+    <hyperlink ref="E136" r:id="rId1" display="https://www.digikey.com/en/products/detail/molex/0039012020/61315?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20234014242&amp;gbraid=0AAAAADrbLlgAu2bzHcOYngWuQW7ztkGxJ&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpl856nujVS8Geug3cuhZcB4DoCpr9xpRmmPa6mjs7ZFHlpXedxvij0aAkumEALw_wcB" xr:uid="{7942DB98-5E6F-4A35-88A4-8452DAD088A7}"/>
+    <hyperlink ref="E106" r:id="rId2" display="https://www.digikey.com/en/products/detail/yageo/RC0603FR-13100RL/12756438?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpn6BH00nvTHufUr9H_-Hg3WEKvE2bn5P98fg2GflffjclQ8k9-V7k4aAmM_EALw_wcB" xr:uid="{CA0412C4-4416-4D1B-B39B-A6DED7EA58CF}"/>
     <hyperlink ref="E16" r:id="rId3" xr:uid="{FDD994C6-E8E1-B746-84DF-96679376034B}"/>
     <hyperlink ref="E17" r:id="rId4" xr:uid="{5128884E-F162-9B46-8FD9-78DFBD3A48A3}"/>
     <hyperlink ref="E32" r:id="rId5" display="https://www.digikey.com/en/products/detail/yageo/CC0603MPY5V9BB104/21285977?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20228387720&amp;gbraid=0AAAAADrbLli2d0istOiCufOq9tFMdO64m&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpkpJxXKr7Hd6DvKJNsC5HlaQ2BA6w4PcrIiTO_QjqzBvssfB6NvXPkaApvXEALw_wcB" xr:uid="{4AC1D765-6997-514E-9B09-03E522CF910A}"/>
@@ -3142,11 +3484,30 @@
     <hyperlink ref="E51" r:id="rId26" xr:uid="{9ED30416-48FE-2F4F-8803-F2E83C003AD6}"/>
     <hyperlink ref="E52" r:id="rId27" xr:uid="{9A03A560-5F50-AD4F-A988-492120C064C8}"/>
     <hyperlink ref="E58" r:id="rId28" display="https://www.google.com/aclk?sa=L&amp;ai=DChsSEwintb_GgKuTAxVsXP8BHekFKZAYACICCAEQCBoCbWQ&amp;ae=2&amp;co=1&amp;ase=2&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKplKIvkp4Z1YOeKEtBTO3lP-fQ4xwLdhiJY9qqgfWdkkFQxFEWYXHjYaAnyzEALw_wcB&amp;cid=CAASugHkaB3vBsMdnevv2CuhrFzshz44TumQCy-zNQeIIxmWWbo9Tk3YXEHFErYg4NFxo2bAMBfbMliGU5Ju6zZdSakRsoGrj9iKH5ub1787B5ItzEEGD0bWd6zAzDuuHkofe1A1zgrpmY6kJpsB_tlMWQ4cJScchvHlcc0vJ5uhgeJ6YRLy1xxK3AzuIfnrOTJMNadrGhb8rPHreEXR7cQBV8EeusF9nV3rW2SIxsVCdCYMoEYeR5Pe-5D-tQk&amp;cce=2&amp;category=acrcp_v1_71&amp;sig=AOD64_08Yaxym_0BKgbLLrQDN-mZAr3AYQ&amp;ctype=5&amp;q=&amp;nis=4&amp;ved=2ahUKEwibo7nGgKuTAxU4kokEHeltMdsQ5bgDKAB6BAgkEAs&amp;adurl=" xr:uid="{14CE9826-7411-8640-BA87-7392C24D2FCF}"/>
-    <hyperlink ref="E65" r:id="rId29" xr:uid="{C798412E-4F32-E34B-B347-E2DF9366383E}"/>
+    <hyperlink ref="E66" r:id="rId29" xr:uid="{C798412E-4F32-E34B-B347-E2DF9366383E}"/>
+    <hyperlink ref="E74" r:id="rId30" display="https://www.digikey.com/en/products/detail/yageo/RC0603FR-1327KL/14287589?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpmK2Nd0C1qZ5MH_NJNoP8nYGRgWf8rHXOeucycBIU26bTpZCW0UCIsaAu_aEALw_wcB" xr:uid="{87928237-1074-364F-974E-A2BE8142D5A3}"/>
+    <hyperlink ref="E75" r:id="rId31" display="https://www.digikey.com/en/products/detail/yageo/RC0603FR-10430RL/14287773?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=17336967819&amp;gbraid=0AAAAADrbLlg549JKDzAotTz6iDuus8fhO&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKplifsrx9xRDrrZ49y-CZCfeUZdf9Dt9xjaYZzNYTq5JgD32A9r3X38aAvbnEALw_wcB" xr:uid="{4C32162B-312B-2B4A-87A7-11B2BFEB593B}"/>
+    <hyperlink ref="E104" r:id="rId32" xr:uid="{F5EC9DC1-859C-3B40-906D-CD491CB2FCB6}"/>
+    <hyperlink ref="E105" r:id="rId33" display="https://www.digikey.com/en/products/detail/yageo/AC0603FR-07499KL/12707691?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpnCMtQRHQvAKmyWuYzA3NNFpFWV7LXez71k_c8RefYnLvEWF7lbSfUaAj3hEALw_wcB" xr:uid="{F8D05555-6BFE-3042-8E27-FE160324420A}"/>
+    <hyperlink ref="E107" r:id="rId34" xr:uid="{7847BBDD-0E09-FC4C-8051-0DE3B5BC7896}"/>
+    <hyperlink ref="E108" r:id="rId35" display="https://www.digikey.com/en/products/detail/stackpole-electronics-inc/RMEF0603FT7K50/16840016?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpnOo1KF7lNez0MbSDEXe3voSS7k8C5CzSx3uagLZW_0-A6xuaswliUaAqm3EALw_wcB" xr:uid="{C4A4FBEC-60D1-5240-843B-4E870F1F98B2}"/>
+    <hyperlink ref="E109" r:id="rId36" display="https://www.digikey.com/en/products/detail/yageo/RC0603FR-072K7P/22199799?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpmWmelQm2ohJMo5u3qcvx9iK8g0JUc6O3suf8zj8fDIxuphuV-rqUwaApu0EALw_wcB" xr:uid="{C48E603E-C71C-8249-BA5C-867049FD0868}"/>
+    <hyperlink ref="E110" r:id="rId37" display="https://www.digikey.com/en/products/detail/yageo/RC0603FR-13100KL/12756433?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20232005509&amp;gbraid=0AAAAADrbLli5wH1-XUSUYxcx5GZx8nGSB&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpmnBYQdKDA9SVV6zpizIORgSwJRBARtjYGz0GzNLLDUTstHQo1xDbsaAqrpEALw_wcB" xr:uid="{DA3C9902-8629-3343-ACF3-36EBB41C4038}"/>
+    <hyperlink ref="E115" r:id="rId38" xr:uid="{4CC57671-B9D2-CB48-9DF1-4893F8622936}"/>
+    <hyperlink ref="E117" r:id="rId39" display="https://www.digikey.com/en/products/detail/recom-power/R-78K3.3-1.0/18093033?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20509822964&amp;gbraid=0AAAAADrbLlheEw7m516CcOgNq4VR1Lyrr&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpm1cS-B90vS9tGYAfdbQ2EfE0k2CScmQPltrpIpaTDAN7SS6OJa1mwaAsMQEALw_wcB" xr:uid="{347B2426-BD48-DB4A-BFE8-67CE4740D8B9}"/>
+    <hyperlink ref="E118" r:id="rId40" xr:uid="{9819139D-77B1-C24E-86C3-6A356945120A}"/>
+    <hyperlink ref="E119" r:id="rId41" display="https://www.digikey.com/en/products/detail/texas-instruments/SN74LVC1G17DBVRG4/4833886?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20228387720&amp;gbraid=0AAAAADrbLli2d0istOiCufOq9tFMdO64m&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpkgNcRbn1r9VOCY0XXEYU46em3umnznFMRcYvAIqWMq9pytEMw77BwaAivfEALw_wcB" xr:uid="{B4EA0295-9DCE-574B-9EB5-C23777B9041D}"/>
+    <hyperlink ref="E120" r:id="rId42" xr:uid="{69491763-D36C-354F-97D9-DF34366F93B7}"/>
+    <hyperlink ref="E130" r:id="rId43" xr:uid="{9E2022A0-091A-7640-AE3F-95D692FBCCEA}"/>
+    <hyperlink ref="E131" r:id="rId44" xr:uid="{EE3BDB52-0A43-0C47-AE7E-050D241C391F}"/>
+    <hyperlink ref="E132" r:id="rId45" xr:uid="{CC287EF3-4D40-8247-BB90-73E3A8AE259C}"/>
+    <hyperlink ref="E137" r:id="rId46" display="https://www.google.com/aclk?sa=L&amp;ai=DChsSEwji4_jSqKuTAxXbOAgFHeK8OeYYACICCAEQCBoCbWQ&amp;ae=2&amp;co=1&amp;ase=2&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpl-k6ctg8WXehD5UUFDkewhPiu-oilZ4mS4mmlSLGKQBUFXJMNnSXoaAs8aEALw_wcB&amp;cid=CAASugHkaDfxLfEHb4HBnYsrG36tu5hK68e1hCAg8tFT2ZJu8XvUGe6f4Ha3iumyRGIhhF3lDaVUPmVBubz5vAhJWb4-QIbSpAqj8h0OIMstipnlRmWKwB4SArJCSaxMqOv-atype=5&amp;q=&amp;nis=4&amp;ved=2ahUKEwi-qvPSqKuTAxU3l4kEHXGaDhsQ5bgDKAB6BAguEBU&amp;adurl=" xr:uid="{4A57E440-3525-AC49-A7BE-37AD58028E79}"/>
+    <hyperlink ref="E62" r:id="rId47" display="https://www.google.com/aclk?sa=L&amp;ai=DChsSEwji4_jSqKuTAxXbOAgFHeK8OeYYACICCAEQBxoCbWQ&amp;ae=2&amp;co=1&amp;ase=2&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpneNb4y90KfePdVYxzM-wBtVd0GnomKRyMbH-MO1ab_56V__1jVqo0aApuTEALw_wcB&amp;cid=CAASugHkaDfxLfEHb4HBnYsrG36tu5hK68e1hCAg8tFT2ZJu8XvUGe6f4Ha3iumyRGIhhF3lDaVUPmVBubz5vAhJWb4-QIbSpAqj8h0OIMstipnlRmWKwB4SArJCSaxMqOv-rfYacAZrKzcLayfiQ6Y47YWtYUId_RlrQRR2AIfCChtU0PP4EKOP0lZXPwO8WaK0YySpKwe-1rizCk75GJssFAvdjc58PLhdBRijeMq4n8exsbeKrLC3Lls9coY&amp;cce=2&amp;category=acrcp_v1_71&amp;sig=AOD64_0TozM9BIldbgGuc5ZPXstowVR_Qg&amp;ctype=5&amp;q=&amp;nis=4&amp;ved=2ahUKEwi-qvPSqKuTAxU3l4kEHXGaDhsQ5bgDKAB6BAguEAs&amp;adurl=" xr:uid="{712E9415-331D-754A-95BD-193F4E5582E2}"/>
+    <hyperlink ref="E59" r:id="rId48" display="https://www.digikey.com/en/products/detail/amphenol-icc-fci-/10129378-902002BLF/7915925?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=17336967819&amp;gbraid=0AAAAADrbLlg549JKDzAotTz6iDuus8fhO&amp;gclid=Cj0KCQjwmunNBhDbARIsAOndKpkHOQyEPffp8JdXQRfXV91-LJqn_ypURrMfKfH1KaiVOwHMU6zuULwaAsTvEALw_wcB" xr:uid="{0033FAD2-1665-DE4B-9E77-62489FAE53A1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId30"/>
+    <tablePart r:id="rId49"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated BOM and finished orders
</commit_message>
<xml_diff>
--- a/BOMs/master_BOM.xlsx
+++ b/BOMs/master_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcoyaipen/Documents/GitHub/RGA_Boards/BOMs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Desktop\ECE 4014\RGA\RGA_Boards\BOMs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8E229C4-9E1F-D146-A12C-CF3207BE8005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98E4C77-F711-4D70-AE32-004AD49900D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="243">
   <si>
     <t>Ref</t>
   </si>
@@ -545,9 +545,6 @@
     <t xml:space="preserve">https://www.digikey.com/en/products/detail/kemet/C0603C102K5RACTU/411081 </t>
   </si>
   <si>
-    <t>should I get 4.7nf????</t>
-  </si>
-  <si>
     <t xml:space="preserve">Joseph is greedy https://www.digikey.com/en/products/detail/walsin-technology-corporation/0603N680J500CT/9355039 </t>
   </si>
   <si>
@@ -647,9 +644,6 @@
     <t>https://www.digikey.com/en/products/detail/yageo/RC0603FR-07560RL/727304</t>
   </si>
   <si>
-    <t>None avaiable on digikey</t>
-  </si>
-  <si>
     <t>https://www.digikey.com/en/products/detail/yageo/RC0603JR-070RL/726675</t>
   </si>
   <si>
@@ -741,13 +735,43 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/molex/0436450310/7062847?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20234014242&amp;gbraid=0AAAAADrbLlgAu2bzHcOYngWuQW7ztkGxJ</t>
+  </si>
+  <si>
+    <t>Chud Marco will get 499 k ohm resistors</t>
+  </si>
+  <si>
+    <t>4.7nf</t>
+  </si>
+  <si>
+    <t>We can take these from the senior design shop</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Molex/76829-0004?qs=KpdAywxU0120juwtNw8Xjw%3D%3D</t>
+  </si>
+  <si>
+    <t>also got mate: https://www.mouser.com/ProductDetail/Molex/170001-0104?qs=MxnWX8BLHKfaXqdKbFiMEg%3D%3D</t>
+  </si>
+  <si>
+    <t>Molex_Mini-Fit_Jr_5566-02A_2x01_P4.20mm_Vertical</t>
+  </si>
+  <si>
+    <t>We have these already</t>
+  </si>
+  <si>
+    <t>We have this already</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/AD5290YRMZ50-R7/1217962</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/analog-devices-inc/AD5160BRJZ10-RL7/652799</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -794,6 +818,12 @@
     <font>
       <sz val="12"/>
       <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -853,7 +883,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -865,6 +895,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="4"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -1176,22 +1207,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A9:F141"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="30.5" customWidth="1"/>
-    <col min="3" max="3" width="33.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.1640625" customWidth="1"/>
+    <col min="1" max="2" width="30.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.77734375" customWidth="1"/>
+    <col min="4" max="4" width="28.109375" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
-    <col min="6" max="6" width="75.5" customWidth="1"/>
+    <col min="6" max="6" width="75.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>145</v>
       </c>
       <c r="B9" s="4"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
@@ -1211,7 +1242,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:6" s="6" customFormat="1" ht="14" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" s="6" customFormat="1" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>89</v>
       </c>
@@ -1231,7 +1262,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="17" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>89</v>
       </c>
@@ -1251,7 +1282,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="18" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>89</v>
       </c>
@@ -1271,29 +1302,32 @@
         <v>163</v>
       </c>
     </row>
-    <row r="19" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
+    <row r="19" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="7">
-        <v>1</v>
-      </c>
-      <c r="D19" s="7" t="s">
+      <c r="B19" s="6">
+        <v>10</v>
+      </c>
+      <c r="C19" s="6">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="F19" s="6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>89</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C20" s="6">
         <v>1</v>
@@ -1305,7 +1339,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="21" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>89</v>
       </c>
@@ -1325,7 +1359,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="22" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>89</v>
       </c>
@@ -1345,7 +1379,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="23" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>89</v>
       </c>
@@ -1365,7 +1399,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="24" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>89</v>
       </c>
@@ -1385,7 +1419,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="25" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>89</v>
       </c>
@@ -1405,7 +1439,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="26" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>89</v>
       </c>
@@ -1422,10 +1456,10 @@
         <v>118</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>89</v>
       </c>
@@ -1439,13 +1473,13 @@
         <v>107</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F27" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="28" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>89</v>
       </c>
@@ -1462,10 +1496,10 @@
         <v>119</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
         <v>89</v>
       </c>
@@ -1485,7 +1519,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="30" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>89</v>
       </c>
@@ -1505,7 +1539,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="31" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>89</v>
       </c>
@@ -1525,12 +1559,12 @@
         <v>163</v>
       </c>
     </row>
-    <row r="32" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="6" t="s">
         <v>89</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C32" s="6">
         <v>37</v>
@@ -1545,7 +1579,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="33" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>89</v>
       </c>
@@ -1562,10 +1596,10 @@
         <v>123</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
         <v>89</v>
       </c>
@@ -1585,7 +1619,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="35" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>89</v>
       </c>
@@ -1599,13 +1633,13 @@
         <v>5</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F35" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="36" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>89</v>
       </c>
@@ -1619,13 +1653,13 @@
         <v>47</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="37" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>89</v>
       </c>
@@ -1639,13 +1673,13 @@
         <v>45</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="38" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
         <v>134</v>
       </c>
@@ -1665,7 +1699,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="39" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" s="6" t="s">
         <v>134</v>
       </c>
@@ -1679,7 +1713,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="40" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="6" t="s">
         <v>134</v>
       </c>
@@ -1693,13 +1727,13 @@
         <v>48</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="41" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="6" t="s">
         <v>134</v>
       </c>
@@ -1713,13 +1747,13 @@
         <v>90</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F41" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="42" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>143</v>
       </c>
@@ -1739,7 +1773,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="43" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B43" s="6">
         <v>25</v>
       </c>
@@ -1747,16 +1781,16 @@
         <v>11</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F43" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="44" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>135</v>
       </c>
@@ -1767,7 +1801,7 @@
         <v>11</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>29</v>
@@ -1776,7 +1810,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="45" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>135</v>
       </c>
@@ -1790,13 +1824,13 @@
         <v>9</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F45" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="46" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>135</v>
       </c>
@@ -1807,16 +1841,16 @@
         <v>4</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="47" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B47" s="6">
         <v>8</v>
       </c>
@@ -1824,16 +1858,16 @@
         <v>4</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F47" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="48" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>135</v>
       </c>
@@ -1847,41 +1881,47 @@
         <v>10</v>
       </c>
       <c r="E48" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C49" s="6">
+        <v>1</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="F48" s="6" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A49" s="7" t="s">
+    </row>
+    <row r="50" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C49" s="7">
-        <v>1</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F49" s="7" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>135</v>
-      </c>
-      <c r="C50">
+      <c r="B50" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C50" s="6">
         <v>3</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="F50" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="F50" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="9" t="s">
         <v>135</v>
       </c>
@@ -1901,7 +1941,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="52" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A52" s="6" t="s">
         <v>135</v>
       </c>
@@ -1921,7 +1961,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="53" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B53" s="6">
         <v>4</v>
       </c>
@@ -1932,14 +1972,16 @@
         <v>2064610800</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B54" s="3"/>
+      <c r="B54" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="C54" s="3">
         <v>1</v>
       </c>
@@ -1951,66 +1993,81 @@
         <v>163</v>
       </c>
     </row>
-    <row r="55" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A55" s="7" t="s">
+    <row r="55" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C55" s="7">
-        <v>1</v>
-      </c>
-      <c r="D55" s="7" t="s">
+      <c r="B55" s="6">
+        <v>3</v>
+      </c>
+      <c r="C55" s="6">
+        <v>1</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="F55" s="7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="7" t="s">
+      <c r="E55" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A56" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C56" s="7">
+      <c r="B56" s="6">
+        <v>4</v>
+      </c>
+      <c r="C56" s="6">
         <v>2</v>
       </c>
-      <c r="D56" s="7" t="s">
+      <c r="D56" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="F56" s="7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A57" s="7" t="s">
+      <c r="F56" s="6" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C57" s="7">
-        <v>1</v>
-      </c>
-      <c r="D57" s="7" t="s">
+      <c r="B57" s="6">
+        <v>2</v>
+      </c>
+      <c r="C57" s="6">
+        <v>1</v>
+      </c>
+      <c r="D57" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="F57" s="7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A58" s="7" t="s">
+      <c r="F57" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A58" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C58" s="7">
-        <v>1</v>
-      </c>
-      <c r="D58" s="7" t="s">
+      <c r="B58" s="6">
+        <v>2</v>
+      </c>
+      <c r="C58" s="6">
+        <v>1</v>
+      </c>
+      <c r="D58" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E58" s="7" t="s">
+      <c r="E58" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="F58" s="7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="F58" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
         <v>135</v>
       </c>
@@ -2030,7 +2087,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="60" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
         <v>135</v>
       </c>
@@ -2050,7 +2107,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="61" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B61" s="6">
         <v>10</v>
       </c>
@@ -2061,10 +2118,10 @@
         <v>113</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
         <v>135</v>
       </c>
@@ -2084,21 +2141,24 @@
         <v>163</v>
       </c>
     </row>
-    <row r="63" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A63" s="9" t="s">
+    <row r="63" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C63" s="9">
+      <c r="B63" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C63" s="6">
         <v>3</v>
       </c>
-      <c r="D63" s="9" t="s">
+      <c r="D63" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F63" s="9" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="F63" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>140</v>
       </c>
@@ -2112,13 +2172,13 @@
         <v>65</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="65" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>140</v>
       </c>
@@ -2132,13 +2192,13 @@
         <v>66</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F65" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="66" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
         <v>140</v>
       </c>
@@ -2158,7 +2218,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="67" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>139</v>
       </c>
@@ -2172,16 +2232,19 @@
         <v>50</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F67" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="68" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="B68" s="9" t="s">
+        <v>176</v>
+      </c>
       <c r="C68" s="9">
         <v>2</v>
       </c>
@@ -2189,14 +2252,16 @@
         <v>71</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B69" s="3"/>
+      <c r="B69" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="C69" s="3">
         <v>4</v>
       </c>
@@ -2208,7 +2273,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="70" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>139</v>
       </c>
@@ -2222,16 +2287,19 @@
         <v>92</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="71" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="B71" s="9" t="s">
+        <v>176</v>
+      </c>
       <c r="C71" s="9">
         <v>2</v>
       </c>
@@ -2239,13 +2307,16 @@
         <v>93</v>
       </c>
       <c r="F71" s="9" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A72" s="9" t="s">
         <v>139</v>
       </c>
+      <c r="B72" s="9" t="s">
+        <v>176</v>
+      </c>
       <c r="C72" s="9">
         <v>2</v>
       </c>
@@ -2253,24 +2324,27 @@
         <v>94</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A73" s="7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" s="11" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A73" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="C73" s="7">
-        <v>1</v>
-      </c>
-      <c r="D73" s="7" t="s">
+      <c r="B73" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="C73" s="11">
+        <v>1</v>
+      </c>
+      <c r="D73" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="F73" s="7" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="F73" s="11" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>67</v>
       </c>
@@ -2290,7 +2364,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="75" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>67</v>
       </c>
@@ -2310,7 +2384,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="76" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>67</v>
       </c>
@@ -2327,10 +2401,10 @@
         <v>32</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>67</v>
       </c>
@@ -2350,7 +2424,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="78" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>67</v>
       </c>
@@ -2370,7 +2444,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="79" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>67</v>
       </c>
@@ -2390,7 +2464,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="80" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>67</v>
       </c>
@@ -2410,7 +2484,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="81" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
         <v>67</v>
       </c>
@@ -2424,13 +2498,13 @@
         <v>51</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F81" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="82" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>67</v>
       </c>
@@ -2444,10 +2518,10 @@
         <v>53</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
         <v>67</v>
       </c>
@@ -2461,13 +2535,13 @@
         <v>54</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F83" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="84" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>67</v>
       </c>
@@ -2481,13 +2555,13 @@
         <v>55</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="85" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
         <v>67</v>
       </c>
@@ -2501,41 +2575,47 @@
         <v>560</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F85" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="86" spans="1:6" s="7" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A86" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C86" s="7">
+    <row r="86" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B86" s="6">
+        <v>20</v>
+      </c>
+      <c r="C86" s="6">
         <v>4</v>
       </c>
-      <c r="D86" s="7" t="s">
+      <c r="D86" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="F86" s="7" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A87" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C87" s="9">
+      <c r="F86" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A87" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B87" s="6">
+        <v>10</v>
+      </c>
+      <c r="C87" s="6">
         <v>2</v>
       </c>
-      <c r="D87" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="F87" s="9" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="D87" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>67</v>
       </c>
@@ -2549,13 +2629,13 @@
         <v>0</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="89" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A89" s="6" t="s">
         <v>67</v>
       </c>
@@ -2569,13 +2649,13 @@
         <v>74</v>
       </c>
       <c r="E89" s="6" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F89" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
         <v>67</v>
       </c>
@@ -2589,13 +2669,13 @@
         <v>75</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="91" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A91" s="6" t="s">
         <v>67</v>
       </c>
@@ -2609,13 +2689,13 @@
         <v>76</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F91" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A92" s="6" t="s">
         <v>67</v>
       </c>
@@ -2629,13 +2709,13 @@
         <v>77</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F92" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="93" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A93" s="6" t="s">
         <v>67</v>
       </c>
@@ -2649,13 +2729,13 @@
         <v>79</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F93" s="9" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>67</v>
       </c>
@@ -2669,13 +2749,13 @@
         <v>72</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A95" s="6" t="s">
         <v>67</v>
       </c>
@@ -2689,13 +2769,13 @@
         <v>83</v>
       </c>
       <c r="E95" s="6" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F95" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="96" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A96" s="6" t="s">
         <v>67</v>
       </c>
@@ -2709,13 +2789,13 @@
         <v>84</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="97" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A97" s="6" t="s">
         <v>67</v>
       </c>
@@ -2729,13 +2809,13 @@
         <v>85</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F97" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A98" s="6" t="s">
         <v>67</v>
       </c>
@@ -2749,13 +2829,13 @@
         <v>86</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A99" s="6" t="s">
         <v>67</v>
       </c>
@@ -2769,13 +2849,13 @@
         <v>73</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="F99" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A100" s="6" t="s">
         <v>67</v>
       </c>
@@ -2789,13 +2869,13 @@
         <v>87</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A101" s="6" t="s">
         <v>67</v>
       </c>
@@ -2809,13 +2889,13 @@
         <v>78</v>
       </c>
       <c r="E101" s="6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F101" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A102" s="6" t="s">
         <v>67</v>
       </c>
@@ -2829,13 +2909,13 @@
         <v>510</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A103" s="6" t="s">
         <v>67</v>
       </c>
@@ -2849,13 +2929,13 @@
         <v>57</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F103" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="104" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A104" s="6" t="s">
         <v>67</v>
       </c>
@@ -2875,7 +2955,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A105" s="6" t="s">
         <v>67</v>
       </c>
@@ -2895,7 +2975,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
         <v>67</v>
       </c>
@@ -2915,7 +2995,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A107" s="6" t="s">
         <v>67</v>
       </c>
@@ -2929,13 +3009,13 @@
         <v>115</v>
       </c>
       <c r="E107" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="F107" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A108" s="6" t="s">
         <v>67</v>
       </c>
@@ -2955,7 +3035,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A109" s="6" t="s">
         <v>67</v>
       </c>
@@ -2975,7 +3055,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="110" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A110" s="6" t="s">
         <v>67</v>
       </c>
@@ -2995,7 +3075,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="111" spans="1:6" s="9" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" s="9" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A111" s="9" t="s">
         <v>67</v>
       </c>
@@ -3012,24 +3092,27 @@
         <v>147</v>
       </c>
       <c r="F111" s="9" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A112" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C112">
-        <v>1</v>
-      </c>
-      <c r="D112" t="s">
+      <c r="B112" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C112" s="6">
+        <v>1</v>
+      </c>
+      <c r="D112" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F112" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="F112" s="6" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A113" s="6" t="s">
         <v>137</v>
       </c>
@@ -3043,27 +3126,30 @@
         <v>18</v>
       </c>
       <c r="E113" s="6" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="F113" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
+    <row r="114" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A114" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C114">
-        <v>1</v>
-      </c>
-      <c r="D114" t="s">
+      <c r="B114" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C114" s="6">
+        <v>1</v>
+      </c>
+      <c r="D114" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F114" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="F114" s="6" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A115" s="6" t="s">
         <v>137</v>
       </c>
@@ -3083,7 +3169,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="116" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A116" s="6" t="s">
         <v>138</v>
       </c>
@@ -3097,13 +3183,13 @@
         <v>21</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F116" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="117" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A117" s="6" t="s">
         <v>138</v>
       </c>
@@ -3123,7 +3209,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="118" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A118" s="6" t="s">
         <v>138</v>
       </c>
@@ -3140,10 +3226,10 @@
         <v>39</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A119" s="6" t="s">
         <v>138</v>
       </c>
@@ -3163,7 +3249,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A120" s="6" t="s">
         <v>138</v>
       </c>
@@ -3180,10 +3266,10 @@
         <v>41</v>
       </c>
       <c r="F120" s="9" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A121" s="6" t="s">
         <v>138</v>
       </c>
@@ -3197,13 +3283,13 @@
         <v>59</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F121" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="122" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A122" s="6" t="s">
         <v>138</v>
       </c>
@@ -3217,13 +3303,13 @@
         <v>61</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="123" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A123" s="6" t="s">
         <v>138</v>
       </c>
@@ -3237,17 +3323,19 @@
         <v>62</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="F123" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="B124" s="5"/>
+      <c r="B124" s="5" t="s">
+        <v>176</v>
+      </c>
       <c r="C124" s="5">
         <v>1</v>
       </c>
@@ -3259,11 +3347,13 @@
         <v>163</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B125" s="3"/>
+      <c r="B125" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="C125" s="3">
         <v>1</v>
       </c>
@@ -3275,21 +3365,27 @@
         <v>163</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
+    <row r="126" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A126" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C126">
-        <v>1</v>
-      </c>
-      <c r="D126" t="s">
+      <c r="B126" s="6">
+        <v>2</v>
+      </c>
+      <c r="C126" s="6">
+        <v>1</v>
+      </c>
+      <c r="D126" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="F126" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="E126" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="F126" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A127" s="6" t="s">
         <v>138</v>
       </c>
@@ -3303,27 +3399,33 @@
         <v>81</v>
       </c>
       <c r="E127" s="6" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="F127" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
+    <row r="128" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A128" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C128">
-        <v>1</v>
-      </c>
-      <c r="D128" t="s">
+      <c r="B128" s="6">
+        <v>2</v>
+      </c>
+      <c r="C128" s="6">
+        <v>1</v>
+      </c>
+      <c r="D128" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F128" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="E128" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="F128" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
         <v>138</v>
       </c>
@@ -3337,13 +3439,13 @@
         <v>95</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F129" s="6" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
         <v>138</v>
       </c>
@@ -3360,10 +3462,10 @@
         <v>105</v>
       </c>
       <c r="F130" s="6" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A131" s="6" t="s">
         <v>138</v>
       </c>
@@ -3383,7 +3485,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A132" s="6" t="s">
         <v>138</v>
       </c>
@@ -3403,22 +3505,22 @@
         <v>163</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F133" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F134" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F135" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E136" s="2" t="s">
         <v>133</v>
       </c>
@@ -3426,30 +3528,30 @@
         <v>163</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E137" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F137" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F138" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F139" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F140" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="F141" t="s">
         <v>163</v>
       </c>

</xml_diff>